<commit_message>
First try at serial commands from psychopy to control POV
</commit_message>
<xml_diff>
--- a/PsychoPy code (PC computer)/setup_data/trials.xlsx
+++ b/PsychoPy code (PC computer)/setup_data/trials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\goodm\OneDrive\Documents\Saccadic-POV\PsychoPy code (PC computer)\setup_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{AA5DDD17-5B6C-4CB4-A0BE-0A59ECEAC86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1167BA39-8D86-4A36-84F2-97B6DB873D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5370" yWindow="4215" windowWidth="30645" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12285" yWindow="4035" windowWidth="18795" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
   <si>
     <t>forest_letter</t>
   </si>
@@ -40,12 +40,6 @@
   </si>
   <si>
     <t>L</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>H</t>
   </si>
   <si>
     <t>X</t>
@@ -424,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -465,153 +459,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>12</v>
-      </c>
-      <c r="B14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>14</v>
-      </c>
-      <c r="B16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>15</v>
-      </c>
-      <c r="B17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -626,12 +477,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -745,6 +590,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -755,21 +606,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -785,6 +621,21 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
   <ds:schemaRefs>

</xml_diff>